<commit_message>
feat(test): update manual test skill with strict rules and result comparison
</commit_message>
<xml_diff>
--- a/test tesrer ctn.xlsx
+++ b/test tesrer ctn.xlsx
@@ -27,11 +27,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
   <si>
     <t>TC ID</t>
   </si>
   <si>
+    <t>name</t>
+  </si>
+  <si>
     <t>Description</t>
   </si>
   <si>
@@ -45,6 +48,9 @@
   </si>
   <si>
     <t xml:space="preserve">Ghi chú </t>
+  </si>
+  <si>
+    <t>check link</t>
   </si>
   <si>
     <t>Kiểm tra link truy cập web</t>
@@ -58,7 +64,10 @@
 diện website hoàn chỉnh</t>
   </si>
   <si>
-    <t>Nếu có lỗi -&gt;kết thúc</t>
+    <t>Nếu có lỗi -&gt;kết thúc testcase</t>
+  </si>
+  <si>
+    <t>check login</t>
   </si>
   <si>
     <t>Kiểm tra đăng nhập</t>
@@ -69,14 +78,16 @@
   </si>
   <si>
     <t>1. Click nút đăng nhập
-2. Đăng nhập tên tài khoản tester02
-và mật khẩu: 12345678</t>
+2. Đăng nhập tên tài khoản:unknow và mật khẩu:12345678</t>
   </si>
   <si>
     <t>Hiển hiện giao diện dashboard</t>
   </si>
   <si>
-    <t>Tài khoản chưa tồn tại -&gt; Tiến hành thực hiện TC 3 trước</t>
+    <t>Tài khoản chưa tồn tại -&gt; kết thúc testcase</t>
+  </si>
+  <si>
+    <t>check register</t>
   </si>
   <si>
     <t>Kiểm tra đăng ký</t>
@@ -95,7 +106,10 @@
 sang giao diện đăng nhập</t>
   </si>
   <si>
-    <t>Tài khoản đã tồn tại -&gt; ghi lỗi và Kết thúc</t>
+    <t>Tài khoản đã tồn tại -&gt; ghi lỗi và kết thúc testcase</t>
+  </si>
+  <si>
+    <t>check logout</t>
   </si>
   <si>
     <t>Kiểm tra đăng xuất</t>
@@ -111,7 +125,10 @@
     <t xml:space="preserve">Trở về giao diện ban đầu </t>
   </si>
   <si>
-    <t>Có lỗi -&gt; Ghi lỗi và Kết thúc</t>
+    <t>Có lỗi -&gt; ghi lỗi và kết thúc testcase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">check forgot pass </t>
   </si>
   <si>
     <t>Kiểm tra quên mật khẩu</t>
@@ -122,6 +139,9 @@
   </si>
   <si>
     <t>Trả về "Reset link sent to email (check console)"</t>
+  </si>
+  <si>
+    <t>Có lỗi -&gt; Ghi lỗi và kết thúc testcase</t>
   </si>
 </sst>
 </file>
@@ -1276,17 +1296,17 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
-  <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="5"/>
+  <dimension ref="A1:G12"/>
+  <sheetFormatPr defaultColWidth="12.6296296296296" defaultRowHeight="15.75" customHeight="1" outlineLevelCol="6"/>
   <cols>
-    <col min="2" max="2" width="30.5" customWidth="1"/>
-    <col min="3" max="3" width="31.3333333333333" customWidth="1"/>
-    <col min="4" max="4" width="45.8888888888889" customWidth="1"/>
-    <col min="5" max="5" width="53.4444444444444" customWidth="1"/>
-    <col min="6" max="6" width="43.3796296296296" customWidth="1"/>
+    <col min="2" max="3" width="30.5" customWidth="1"/>
+    <col min="4" max="4" width="31.3333333333333" customWidth="1"/>
+    <col min="5" max="5" width="45.8888888888889" customWidth="1"/>
+    <col min="6" max="6" width="53.4444444444444" customWidth="1"/>
+    <col min="7" max="7" width="61.5555555555556" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="39.75" customHeight="1" spans="1:6">
+    <row r="1" ht="39.75" customHeight="1" spans="1:7">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1302,155 +1322,179 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
     </row>
-    <row r="2" ht="25" customHeight="1" spans="1:6">
+    <row r="2" ht="25" customHeight="1" spans="1:7">
       <c r="A2" s="3">
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
+      <c r="C2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4"/>
       <c r="E2" s="3" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
-    <row r="3" ht="53" customHeight="1" spans="1:6">
+    <row r="3" ht="53" customHeight="1" spans="1:7">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>11</v>
+        <v>12</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>13</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>15</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="4" ht="53" customHeight="1" spans="1:6">
+    <row r="4" ht="53" customHeight="1" spans="1:7">
       <c r="A4" s="3">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>21</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>23</v>
       </c>
     </row>
-    <row r="5" ht="51" customHeight="1" spans="1:6">
+    <row r="5" ht="51" customHeight="1" spans="1:7">
       <c r="A5" s="4">
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
         <v>24</v>
       </c>
+      <c r="C5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G5" t="s">
+        <v>29</v>
+      </c>
     </row>
-    <row r="6" ht="64" customHeight="1" spans="1:6">
+    <row r="6" ht="64" customHeight="1" spans="1:7">
       <c r="A6" s="4">
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>32</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>24</v>
+        <v>33</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>34</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="1:6">
+    <row r="7" customHeight="1" spans="1:7">
       <c r="A7" s="4"/>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>
       <c r="D7" s="4"/>
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
     </row>
-    <row r="8" customHeight="1" spans="1:6">
+    <row r="8" customHeight="1" spans="1:7">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="4"/>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
     </row>
-    <row r="9" customHeight="1" spans="1:6">
+    <row r="9" customHeight="1" spans="1:7">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
     </row>
-    <row r="10" customHeight="1" spans="1:6">
+    <row r="10" customHeight="1" spans="1:7">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="4"/>
       <c r="D10" s="4"/>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
+      <c r="G10" s="4"/>
     </row>
-    <row r="11" customHeight="1" spans="1:6">
+    <row r="11" customHeight="1" spans="1:7">
       <c r="A11" s="4"/>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
       <c r="D11" s="4"/>
       <c r="E11" s="4"/>
       <c r="F11" s="4"/>
+      <c r="G11" s="4"/>
     </row>
-    <row r="12" customHeight="1" spans="1:6">
+    <row r="12" customHeight="1" spans="1:7">
       <c r="A12" s="4"/>
       <c r="B12" s="4"/>
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
       <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
test(qabot): update manual test recordings and reports
</commit_message>
<xml_diff>
--- a/test tesrer ctn.xlsx
+++ b/test tesrer ctn.xlsx
@@ -78,7 +78,7 @@
   </si>
   <si>
     <t>1. Click nút đăng nhập
-2. Đăng nhập tên tài khoản:unknow và mật khẩu:12345678</t>
+2. Đăng nhập tên tài khoản:unknow1 và mật khẩu:12345678</t>
   </si>
   <si>
     <t>Hiển hiện giao diện dashboard</t>
@@ -98,7 +98,7 @@
   <si>
     <t>1. Click nút đăng ký
 2. Đăng ký với tài khoản tester02
-3. email. tester02@gmail.com
+3. email:tester02@gmail.com
 4. mật khẩu: 12345678</t>
   </si>
   <si>

</xml_diff>

<commit_message>
feat(automation): upgrade to AI Automation Suite v2 with isolated storage and timestamping
</commit_message>
<xml_diff>
--- a/test tesrer ctn.xlsx
+++ b/test tesrer ctn.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9120"/>
+    <workbookView windowWidth="23040" windowHeight="8400"/>
   </bookViews>
   <sheets>
     <sheet name="Trang tính1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
   <si>
     <t>TC ID</t>
   </si>
@@ -73,65 +73,69 @@
     <t>Kiểm tra đăng nhập</t>
   </si>
   <si>
+    <t xml:space="preserve">server đã chạy
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+ Đăng nhập tên tài khoản:"ctn" và mật khẩu:"12345678"</t>
+  </si>
+  <si>
+    <t>Hiển hiện giao diện dashboard</t>
+  </si>
+  <si>
+    <t>Tài khoản chưa tồn tại -&gt; kết thúc testcase</t>
+  </si>
+  <si>
+    <t>check register</t>
+  </si>
+  <si>
+    <t>Kiểm tra đăng ký</t>
+  </si>
+  <si>
+    <t>Link server web đã tồn tại.</t>
+  </si>
+  <si>
+    <t>1. Click nút đăng ký
+2. Đăng ký với tài khoản "tester11"
+3. email:"tester11@gmail.com"
+4. mật khẩu:"12345678"</t>
+  </si>
+  <si>
+    <t>Đăng ký thành công và chuyển 
+sang giao diện đăng nhập</t>
+  </si>
+  <si>
+    <t>Tài khoản đã tồn tại -&gt; ghi lỗi và kết thúc testcase</t>
+  </si>
+  <si>
+    <t>check logout</t>
+  </si>
+  <si>
+    <t>Kiểm tra đăng xuất</t>
+  </si>
+  <si>
+    <t>Đăng nhập thành công</t>
+  </si>
+  <si>
+    <t>Đăng nhập bằng tài khoản và mật khẩu ở TC 3
+click logout</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trở về giao diện ban đầu </t>
+  </si>
+  <si>
+    <t>Có lỗi -&gt; ghi lỗi và kết thúc testcase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">check forgot pass </t>
+  </si>
+  <si>
+    <t>Kiểm tra quên mật khẩu</t>
+  </si>
+  <si>
     <t xml:space="preserve"> Link server web đã tồn tại.
 </t>
-  </si>
-  <si>
-    <t>1. Click nút đăng nhập
-2. Đăng nhập tên tài khoản:unknow1 và mật khẩu:12345678</t>
-  </si>
-  <si>
-    <t>Hiển hiện giao diện dashboard</t>
-  </si>
-  <si>
-    <t>Tài khoản chưa tồn tại -&gt; kết thúc testcase</t>
-  </si>
-  <si>
-    <t>check register</t>
-  </si>
-  <si>
-    <t>Kiểm tra đăng ký</t>
-  </si>
-  <si>
-    <t>Link server web đã tồn tại.</t>
-  </si>
-  <si>
-    <t>1. Click nút đăng ký
-2. Đăng ký với tài khoản tester02
-3. email:tester02@gmail.com
-4. mật khẩu: 12345678</t>
-  </si>
-  <si>
-    <t>Đăng ký thành công và chuyển 
-sang giao diện đăng nhập</t>
-  </si>
-  <si>
-    <t>Tài khoản đã tồn tại -&gt; ghi lỗi và kết thúc testcase</t>
-  </si>
-  <si>
-    <t>check logout</t>
-  </si>
-  <si>
-    <t>Kiểm tra đăng xuất</t>
-  </si>
-  <si>
-    <t>Đăng nhập thành công</t>
-  </si>
-  <si>
-    <t>Đăng nhập bằng tài khoản và mật khẩu ở TC 2
-click logout</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Trở về giao diện ban đầu </t>
-  </si>
-  <si>
-    <t>Có lỗi -&gt; ghi lỗi và kết thúc testcase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">check forgot pass </t>
-  </si>
-  <si>
-    <t>Kiểm tra quên mật khẩu</t>
   </si>
   <si>
     <t>1. Click Forgot Password
@@ -1430,16 +1434,16 @@
         <v>31</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" customHeight="1" spans="1:7">

</xml_diff>